<commit_message>
updated xlwings version to fix plotting
</commit_message>
<xml_diff>
--- a/lite/weather.xlsx
+++ b/lite/weather.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10331"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10625"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/felix/dev/python-for-excel/lite/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{281C4CC4-A0C8-264E-BA36-5BDFC45429BC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9FAE3E0-9091-974C-A73D-589693193252}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="880" yWindow="780" windowWidth="33320" windowHeight="21360" xr2:uid="{BEEA179C-679E-224E-B4F3-A66533203FCC}"/>
   </bookViews>
@@ -478,10 +478,13 @@
   <we:properties>
     <we:property name="main.py" value="&quot;import datetime as dt\n\nimport matplotlib.pyplot as plt\nimport pandas as pd\nimport requests\nfrom xlwings import arg, func, ret\n\n\n@func\n@ret(index=False)\ndef get_temperature_history(\n    latitude: float,\n    longitude: float,\n    start_date: dt.date,\n    end_date: dt.date,\n):\n    # Open-Meteo API for historical data\n    url = \&quot;https:\/\/archive-api.open-meteo.com\/v1\/archive\&quot;\n\n    # Making the web API request\n    params = {\n        \&quot;latitude\&quot;: latitude,\n        \&quot;longitude\&quot;: longitude,\n        \&quot;daily\&quot;: \&quot;temperature_2m_min,temperature_2m_max\&quot;,\n        \&quot;start_date\&quot;: start_date.isoformat(),\n        \&quot;end_date\&quot;: end_date.isoformat(),\n        \&quot;temperature_unit\&quot;: \&quot;fahrenheit\&quot;,\n        \&quot;timezone\&quot;: \&quot;auto\&quot;,\n    }\n    response = requests.get(url, params=params)\n    response.raise_for_status()\n    data = response.json()\n\n    # Turn the data into a DataFrame to easily return it to Excel\n    df = pd.DataFrame(\n        {\n            \&quot;Date\&quot;: pd.to_datetime(data[\&quot;daily\&quot;][\&quot;time\&quot;]),\n            \&quot;Min. Temperature (°F)\&quot;: data[\&quot;daily\&quot;][\&quot;temperature_2m_min\&quot;],\n            \&quot;Max. Temperature (°F)\&quot;: data[\&quot;daily\&quot;][\&quot;temperature_2m_max\&quot;],\n        }\n    )\n\n    return df\n\n\n@func\n@arg(\&quot;df\&quot;, parse_dates=[\&quot;Date\&quot;])\ndef plot_temperature(df: pd.DataFrame):\n    # Create a figure and axes object to be able to create a secondary axis\n    fig, ax = plt.subplots(figsize=(8, 5))\n\n    # Plotting min. and max. temperature\n    df[\&quot;Min. Temperature (°F)\&quot;].plot(ax=ax, color=\&quot;blue\&quot;, label=\&quot;Min Temp\&quot;)\n    df[\&quot;Max. Temperature (°F)\&quot;].plot(ax=ax, color=\&quot;red\&quot;, label=\&quot;Max Temp\&quot;)\n\n    # Secondary Y-axis for Celsius\n    def f_to_c(x):\n        return (x - 32) * 5 \/ 9\n\n    def c_to_f(x):\n        return x * 9 \/ 5 + 32\n\n    secax = ax.secondary_yaxis(\&quot;right\&quot;, functions=(f_to_c, c_to_f))\n\n    # Formatting\n    ax.set_title(\&quot;Daily Min and Max Temperatures\&quot;, fontsize=14)\n    ax.set_xlabel(\&quot;Date\&quot;, fontsize=14)\n    ax.set_ylabel(\&quot;Temperature (°F)\&quot;, fontsize=14)\n    secax.set_ylabel(\&quot;Temperature (°C)\&quot;, fontsize=14)\n    ax.minorticks_off()\n    ax.grid(alpha=0.5)\n    ax.legend()\n\n    return fig\n&quot;"/>
     <we:property name="pyodideVersion" value="&quot;0.27.5&quot;"/>
-    <we:property name="addinVersion" value="&quot;1.0.0.0-19&quot;"/>
-    <we:property name="requirements.txt" value="&quot;# Pin the version of packages that are installed from PyPI.\n# Don't pin the version if they are on this list:\n# https:\/\/pyodide.org\/en\/stable\/usage\/packages-in-pyodide.html\n#\n# New packages are installed on the fly.\n# However, the following situations require a restart:\n# - removing a package\n# - changing the version of a package\n# - adding an optional dependency of xlwings, e.g, polars\n\nxlwings==0.33.19  # required\npython-dotenv==1.2.1  # required\npyodide-http  # required\nblack  # required\npandas\nmatplotlib\nrequests&quot;"/>
+    <we:property name="addinVersion" value="&quot;1.0.0.88&quot;"/>
+    <we:property name="requirements.txt" value="&quot;# Pin the version of packages that are installed from PyPI.\n# Don't pin the version if they are on this list:\n# https:\/\/pyodide.org\/en\/stable\/usage\/packages-in-pyodide.html\n#\n# New packages are installed on the fly.\n# However, the following situations require a restart:\n# - removing a package\n# - changing the version of a package\n# - adding an optional dependency of xlwings, e.g, polars\n\nxlwings==0.36.8  # required\npython-dotenv==1.2.1  # required\npyodide-http  # required\npandas\nmatplotlib\nrequests&quot;"/>
     <we:property name="xlwingsWorkbookId" value="&quot;a9300ad2-41a3-4596-9452-1a01b6e34ebe&quot;"/>
     <we:property name="xlwingsSettingsWorkbook" value="&quot;{\&quot;startupBehavior\&quot;:\&quot;taskpane\&quot;}&quot;"/>
+    <we:property name="notebook.py" value="&quot;&quot;"/>
+    <we:property name="pyproject.toml" value="&quot;# RESTART AFTER MAKING CHANGES\n\n# Ruff: linter &amp; code formatter\n[tool.ruff]\nfix = true\npreview = true\n\n# Ty: type checker &amp; language server\n[tool.ty.rules]\n&quot;"/>
+    <we:property name="tests.py" value="&quot;&quot;"/>
   </we:properties>
   <we:bindings/>
   <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
@@ -491,9 +494,14 @@
     </a:ext>
     <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{7C84B067-C214-45C3-A712-C9D94CD141B2}">
       <we:customFunctionIdList>
-        <we:customFunctionIds>_xldudf_WINGMAN</we:customFunctionIds>
-        <we:customFunctionIds>_xldudf_GET_TEMPERATURE_HISTORY</we:customFunctionIds>
-        <we:customFunctionIds>_xldudf_PLOT_TEMPERATURE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_CORREL2</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_DF_QUERY</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_GET_DF</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_HEATMAP</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_HELLO</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_PLOT_SINE</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_STANDARD_NORMAL</we:customFunctionIds>
+        <we:customFunctionIds>_xldudf_STREAMING_RANDOM</we:customFunctionIds>
       </we:customFunctionIdList>
     </a:ext>
     <a:ext xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" uri="{0858819E-0033-43BF-8937-05EC82904868}">

</xml_diff>